<commit_message>
crossing line and direction counter
</commit_message>
<xml_diff>
--- a/Traffic_Analysis_Log.xlsx
+++ b/Traffic_Analysis_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexander\Documents\.Personal\.School\Binghamton Spring 2025\Traffic-Analysis-Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54765654-0897-43B4-9FC4-E268E2EF45B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D575201-1620-4AA2-BB1E-B1ADB8B52A4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="119">
   <si>
     <t>Filename</t>
   </si>
@@ -261,13 +261,132 @@
     <t>2025-05-07 04:48:21</t>
   </si>
   <si>
+    <t>test for automatic center alignment of data, failed and retroactively fixed</t>
+  </si>
+  <si>
     <t>2025-05-07 04:50:31</t>
   </si>
   <si>
     <t>test for automatic center alignment of data, passed</t>
   </si>
   <si>
-    <t>test for automatic center alignment of data, failed and retroactively fixed</t>
+    <t>2025-05-12 18:57:27</t>
+  </si>
+  <si>
+    <t>lane detection test, failed</t>
+  </si>
+  <si>
+    <t>I-695 at Randall Avenue.mp4</t>
+  </si>
+  <si>
+    <t>2202x1450</t>
+  </si>
+  <si>
+    <t>I-695 Throgs Neck Expressway</t>
+  </si>
+  <si>
+    <t>southbound</t>
+  </si>
+  <si>
+    <t>fog</t>
+  </si>
+  <si>
+    <t>2025-05-12 18:58:59</t>
+  </si>
+  <si>
+    <t>2025-05-12 19:31:56</t>
+  </si>
+  <si>
+    <t>Centroid Tracker + Line Crossing</t>
+  </si>
+  <si>
+    <t>lane detection test, improved
+undercounting vehicles</t>
+  </si>
+  <si>
+    <t>I-695 at Randall Avenue new.mp4</t>
+  </si>
+  <si>
+    <t>cloudy</t>
+  </si>
+  <si>
+    <t>sunset</t>
+  </si>
+  <si>
+    <t>2025-05-12 19:33:38</t>
+  </si>
+  <si>
+    <t>2025-05-12 19:36:21</t>
+  </si>
+  <si>
+    <t>lane detection test, improved
+results likley improved because of higher resolution</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:02:40</t>
+  </si>
+  <si>
+    <t>SORT + Line Crossing</t>
+  </si>
+  <si>
+    <t>SORT tracking test, improved
+still undercounting</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:05:08</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:28:51</t>
+  </si>
+  <si>
+    <t>crossing line bounding box adujstment, slight improvement
+still undercounting</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:30:25</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:39:17</t>
+  </si>
+  <si>
+    <t>DirA/DirB vehicle counting, incorrectly drawn lines</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:46:30</t>
+  </si>
+  <si>
+    <t>DirA/DirB vehicle counting, correctly drawn lines
+bug counting all vehicles under DirB, not logging</t>
+  </si>
+  <si>
+    <t>2025-05-12 20:54:44</t>
+  </si>
+  <si>
+    <t>resolved bug counting all behicles under DirB
+still not logging</t>
+  </si>
+  <si>
+    <t>2025-05-12 21:07:44</t>
+  </si>
+  <si>
+    <t>bug where DirB logging falls under wrong label "VPMPL (DirA_L5)"
+retroactivley fixed with manual entries</t>
+  </si>
+  <si>
+    <t>2025-05-12 21:15:50</t>
+  </si>
+  <si>
+    <t>2025-05-12 21:19:01</t>
+  </si>
+  <si>
+    <t>2025-05-12 21:28:19</t>
+  </si>
+  <si>
+    <t>2025-05-12 21:34:55</t>
+  </si>
+  <si>
+    <t>wrong label logging bug resolved, now correctly logging directional flow
+new bug discovered where some DirB traffic is counted as DirA</t>
   </si>
 </sst>
 </file>
@@ -680,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AY6"/>
+  <dimension ref="A1:AY23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.85546875" style="6" bestFit="1" customWidth="1"/>
@@ -699,7 +818,7 @@
     <col min="14" max="14" width="26.7109375" style="10" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.85546875" style="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.85546875" style="6" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="28.85546875" style="6" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="24.7109375" style="6" bestFit="1" customWidth="1"/>
@@ -727,8 +846,8 @@
     <col min="45" max="45" width="16.140625" style="9" bestFit="1" customWidth="1"/>
     <col min="46" max="46" width="33.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="47" max="51" width="16" style="6" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="9.140625" style="6" customWidth="1"/>
-    <col min="53" max="16384" width="9.140625" style="6"/>
+    <col min="52" max="62" width="9.140625" style="6" customWidth="1"/>
+    <col min="63" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:51" x14ac:dyDescent="0.25">
@@ -886,7 +1005,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:51" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>51</v>
       </c>
@@ -1041,7 +1160,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:51" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>51</v>
       </c>
@@ -1419,7 +1538,7 @@
         <v>0</v>
       </c>
       <c r="W5" s="6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="X5" s="6">
         <v>2423</v>
@@ -1550,7 +1669,7 @@
         <v>77</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="P6" s="6" t="s">
         <v>63</v>
@@ -1574,7 +1693,7 @@
         <v>0</v>
       </c>
       <c r="W6" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="X6" s="6">
         <v>2423</v>
@@ -1658,6 +1777,2641 @@
         <v>53</v>
       </c>
       <c r="AY6" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="6">
+        <v>80.17</v>
+      </c>
+      <c r="D7" s="6">
+        <v>30</v>
+      </c>
+      <c r="E7" s="6">
+        <v>2405</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V7" s="6">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="X7" s="6">
+        <v>568</v>
+      </c>
+      <c r="Y7" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR7" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY7" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="6">
+        <v>90.37</v>
+      </c>
+      <c r="D8" s="6">
+        <v>30</v>
+      </c>
+      <c r="E8" s="6">
+        <v>2711</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="O8" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="P8" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q8" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V8" s="6">
+        <v>0</v>
+      </c>
+      <c r="W8" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="X8" s="6">
+        <v>365</v>
+      </c>
+      <c r="Y8" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI8" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR8" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY8" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="6">
+        <v>90.37</v>
+      </c>
+      <c r="D9" s="6">
+        <v>30</v>
+      </c>
+      <c r="E9" s="6">
+        <v>2711</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V9" s="6">
+        <v>0</v>
+      </c>
+      <c r="W9" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="X9" s="6">
+        <v>24</v>
+      </c>
+      <c r="Y9" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR9" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY9" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D10" s="6">
+        <v>30</v>
+      </c>
+      <c r="E10" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q10" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V10" s="6">
+        <v>0</v>
+      </c>
+      <c r="W10" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="X10" s="6">
+        <v>28</v>
+      </c>
+      <c r="Y10" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR10" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY10" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="6">
+        <v>42.54</v>
+      </c>
+      <c r="D11" s="6">
+        <v>29.97</v>
+      </c>
+      <c r="E11" s="6">
+        <v>1275</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="O11" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q11" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="R11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V11" s="6">
+        <v>0</v>
+      </c>
+      <c r="W11" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="X11" s="6">
+        <v>408</v>
+      </c>
+      <c r="Y11" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR11" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY11" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D12" s="6">
+        <v>30</v>
+      </c>
+      <c r="E12" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N12" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q12" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V12" s="6">
+        <v>0</v>
+      </c>
+      <c r="W12" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="X12" s="6">
+        <v>40</v>
+      </c>
+      <c r="Y12" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR12" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY12" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="6">
+        <v>90.37</v>
+      </c>
+      <c r="D13" s="6">
+        <v>30</v>
+      </c>
+      <c r="E13" s="6">
+        <v>2711</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N13" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="O13" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q13" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V13" s="6">
+        <v>0</v>
+      </c>
+      <c r="W13" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="X13" s="6">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX13" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY13" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" s="6">
+        <v>90.37</v>
+      </c>
+      <c r="D14" s="6">
+        <v>30</v>
+      </c>
+      <c r="E14" s="6">
+        <v>2711</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="O14" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="P14" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V14" s="6">
+        <v>0</v>
+      </c>
+      <c r="W14" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="X14" s="6">
+        <v>28</v>
+      </c>
+      <c r="Y14" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY14" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D15" s="6">
+        <v>30</v>
+      </c>
+      <c r="E15" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q15" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V15" s="6">
+        <v>0</v>
+      </c>
+      <c r="W15" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="X15" s="6">
+        <v>41</v>
+      </c>
+      <c r="Y15" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI15" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR15" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX15" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY15" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:51" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D16" s="6">
+        <v>30</v>
+      </c>
+      <c r="E16" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q16" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V16" s="6">
+        <v>0</v>
+      </c>
+      <c r="W16" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="X16" s="6">
+        <v>41</v>
+      </c>
+      <c r="Y16" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI16" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR16" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX16" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY16" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D17" s="6">
+        <v>30</v>
+      </c>
+      <c r="E17" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K17" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O17" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V17" s="6">
+        <v>0</v>
+      </c>
+      <c r="W17" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="X17" s="6">
+        <v>41</v>
+      </c>
+      <c r="Y17" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI17" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR17" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX17" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY17" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D18" s="6">
+        <v>30</v>
+      </c>
+      <c r="E18" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L18" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M18" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N18" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="P18" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q18" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V18" s="6">
+        <v>0</v>
+      </c>
+      <c r="W18" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="X18" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y18" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI18" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AM18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR18" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX18" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY18" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D19" s="6">
+        <v>30</v>
+      </c>
+      <c r="E19" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O19" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V19" s="6">
+        <v>0</v>
+      </c>
+      <c r="W19" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="X19" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y19" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI19" s="6">
+        <v>41</v>
+      </c>
+      <c r="AJ19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL19" s="6">
+        <v>19</v>
+      </c>
+      <c r="AM19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR19" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX19" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY19" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D20" s="6">
+        <v>30</v>
+      </c>
+      <c r="E20" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="P20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q20" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V20" s="6">
+        <v>0</v>
+      </c>
+      <c r="W20" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="X20" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y20" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI20" s="6">
+        <v>41</v>
+      </c>
+      <c r="AJ20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL20" s="6">
+        <v>19</v>
+      </c>
+      <c r="AM20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR20" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX20" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY20" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D21" s="6">
+        <v>30</v>
+      </c>
+      <c r="E21" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q21" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V21" s="6">
+        <v>0</v>
+      </c>
+      <c r="W21" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="X21" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y21" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI21" s="6">
+        <v>41</v>
+      </c>
+      <c r="AJ21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL21" s="6">
+        <v>19</v>
+      </c>
+      <c r="AM21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR21" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX21" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY21" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:51" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D22" s="6">
+        <v>30</v>
+      </c>
+      <c r="E22" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J22" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L22" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M22" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O22" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="P22" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V22" s="6">
+        <v>0</v>
+      </c>
+      <c r="W22" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="X22" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y22" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI22" s="6">
+        <v>41</v>
+      </c>
+      <c r="AJ22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL22" s="6">
+        <v>19</v>
+      </c>
+      <c r="AM22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR22" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX22" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY22" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:51" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="6">
+        <v>86.83</v>
+      </c>
+      <c r="D23" s="6">
+        <v>30</v>
+      </c>
+      <c r="E23" s="6">
+        <v>2605</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L23" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="M23" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="N23" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="O23" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="P23" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q23" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="R23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="T23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="U23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="V23" s="6">
+        <v>0</v>
+      </c>
+      <c r="W23" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="X23" s="6">
+        <v>60</v>
+      </c>
+      <c r="Y23" s="6">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="6">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="6">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI23" s="6">
+        <v>41</v>
+      </c>
+      <c r="AJ23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AK23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL23" s="6">
+        <v>19</v>
+      </c>
+      <c r="AM23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR23" s="6">
+        <v>0</v>
+      </c>
+      <c r="AS23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AT23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AU23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AV23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AW23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AY23" s="6" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>

<commit_message>
motorcycle speed calculations fixed
</commit_message>
<xml_diff>
--- a/Traffic_Analysis_Log.xlsx
+++ b/Traffic_Analysis_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexander\Documents\.Personal\.School\Binghamton Spring 2025\Traffic-Analysis-Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92DAB058-8EAA-4522-B8F5-A3E4C41EEDE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20FB97CD-6E66-4A96-977E-FC27FF977736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17085" yWindow="-105" windowWidth="17415" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Traffic Analysis Log" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2578" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2596" uniqueCount="181">
   <si>
     <t>Filename</t>
   </si>
@@ -555,6 +555,9 @@
     <t>2025-05-14 07:20:00</t>
   </si>
   <si>
+    <t>moving on to finish speed calculations first, attempt failed</t>
+  </si>
+  <si>
     <t>2025-05-14 07:36:58</t>
   </si>
   <si>
@@ -570,10 +573,13 @@
     <t>2025-05-14 08:12:20</t>
   </si>
   <si>
-    <t>finally logging all speeds</t>
-  </si>
-  <si>
-    <t>moving on to finish speed calculations first, attempt failed</t>
+    <t>finally logging all speeds, but miscalculating motorcycle speeds</t>
+  </si>
+  <si>
+    <t>2025-05-14 08:27:56</t>
+  </si>
+  <si>
+    <t>fixed motorcycle speed calculations</t>
   </si>
 </sst>
 </file>
@@ -960,7 +966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BG56"/>
+  <dimension ref="A1:BG57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55.28515625" style="4" bestFit="1" customWidth="1"/>
@@ -1035,8 +1041,8 @@
     <col min="70" max="70" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="71" max="71" width="14.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="72" max="72" width="21.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="73" max="86" width="9.140625" style="4" customWidth="1"/>
-    <col min="87" max="16384" width="9.140625" style="4"/>
+    <col min="73" max="87" width="9.140625" style="4" customWidth="1"/>
+    <col min="88" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:59" x14ac:dyDescent="0.25">
@@ -9777,7 +9783,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="50" spans="1:59" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:59" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>101</v>
       </c>
@@ -10018,7 +10024,7 @@
         <v>0</v>
       </c>
       <c r="W51" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="X51" s="4">
         <v>6.5103999999999997</v>
@@ -10173,7 +10179,7 @@
         <v>103</v>
       </c>
       <c r="O52" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="P52" s="4" t="s">
         <v>71</v>
@@ -10194,7 +10200,7 @@
         <v>0</v>
       </c>
       <c r="W52" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="X52" s="4">
         <v>6.5103999999999997</v>
@@ -10349,7 +10355,7 @@
         <v>103</v>
       </c>
       <c r="O53" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P53" s="4" t="s">
         <v>71</v>
@@ -10370,7 +10376,7 @@
         <v>0</v>
       </c>
       <c r="W53" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="X53" s="4">
         <v>6.5103999999999997</v>
@@ -10525,7 +10531,7 @@
         <v>103</v>
       </c>
       <c r="O54" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P54" s="4" t="s">
         <v>71</v>
@@ -10546,7 +10552,7 @@
         <v>0</v>
       </c>
       <c r="W54" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="X54" s="4">
         <v>6.5103999999999997</v>
@@ -10701,7 +10707,7 @@
         <v>103</v>
       </c>
       <c r="O55" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P55" s="4" t="s">
         <v>71</v>
@@ -10722,7 +10728,7 @@
         <v>0</v>
       </c>
       <c r="W55" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="X55" s="4">
         <v>6.5103999999999997</v>
@@ -10877,7 +10883,7 @@
         <v>103</v>
       </c>
       <c r="O56" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P56" s="4" t="s">
         <v>71</v>
@@ -10898,7 +10904,7 @@
         <v>0</v>
       </c>
       <c r="W56" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="X56" s="4">
         <v>6.5103999999999997</v>
@@ -11007,6 +11013,182 @@
       </c>
       <c r="BG56" s="4" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="57" spans="1:59" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C57" s="4">
+        <v>86.83</v>
+      </c>
+      <c r="D57" s="4">
+        <v>30</v>
+      </c>
+      <c r="E57" s="4">
+        <v>2605</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I57" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K57" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="L57" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="M57" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="N57" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="O57" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="P57" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q57" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="R57" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="S57" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="U57" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V57" s="4">
+        <v>0</v>
+      </c>
+      <c r="W57" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="X57" s="4">
+        <v>6.5103999999999997</v>
+      </c>
+      <c r="Y57" s="4">
+        <v>41.46</v>
+      </c>
+      <c r="Z57" s="4">
+        <v>60</v>
+      </c>
+      <c r="AA57" s="4">
+        <v>51</v>
+      </c>
+      <c r="AB57" s="4">
+        <v>3</v>
+      </c>
+      <c r="AC57" s="4">
+        <v>6</v>
+      </c>
+      <c r="AD57" s="4">
+        <v>0</v>
+      </c>
+      <c r="AE57" s="4">
+        <v>4.4488000000000003</v>
+      </c>
+      <c r="AF57" s="4">
+        <v>28.33</v>
+      </c>
+      <c r="AG57" s="4">
+        <v>41</v>
+      </c>
+      <c r="AH57" s="4">
+        <v>36</v>
+      </c>
+      <c r="AI57" s="4">
+        <v>2</v>
+      </c>
+      <c r="AJ57" s="4">
+        <v>3</v>
+      </c>
+      <c r="AK57" s="4">
+        <v>0</v>
+      </c>
+      <c r="AL57" s="4">
+        <v>2.0615999999999999</v>
+      </c>
+      <c r="AM57" s="4">
+        <v>13.13</v>
+      </c>
+      <c r="AN57" s="4">
+        <v>19</v>
+      </c>
+      <c r="AO57" s="4">
+        <v>15</v>
+      </c>
+      <c r="AP57" s="4">
+        <v>1</v>
+      </c>
+      <c r="AQ57" s="4">
+        <v>3</v>
+      </c>
+      <c r="AR57" s="4">
+        <v>0</v>
+      </c>
+      <c r="AS57" s="4">
+        <v>9.14</v>
+      </c>
+      <c r="AT57" s="4">
+        <v>10.67</v>
+      </c>
+      <c r="AU57" s="4">
+        <v>10.5</v>
+      </c>
+      <c r="AV57" s="4">
+        <v>9.43</v>
+      </c>
+      <c r="AW57" s="4">
+        <v>0</v>
+      </c>
+      <c r="AX57" s="4">
+        <v>6.42</v>
+      </c>
+      <c r="AY57" s="4">
+        <v>6.42</v>
+      </c>
+      <c r="AZ57" s="4">
+        <v>7.06</v>
+      </c>
+      <c r="BA57" s="4">
+        <v>5.67</v>
+      </c>
+      <c r="BB57" s="4">
+        <v>0</v>
+      </c>
+      <c r="BC57" s="4">
+        <v>14.6</v>
+      </c>
+      <c r="BD57" s="4">
+        <v>14.92</v>
+      </c>
+      <c r="BE57" s="4">
+        <v>13.95</v>
+      </c>
+      <c r="BF57" s="4">
+        <v>13.18</v>
+      </c>
+      <c r="BG57" s="4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>